<commit_message>
Added Selenium test report
</commit_message>
<xml_diff>
--- a/react_web_tests/test_report.xlsx
+++ b/react_web_tests/test_report.xlsx
@@ -707,7 +707,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Generated: 2026-06-11 14:55:25   |   App URL: http://localhost:5173</t>
+          <t xml:space="preserve">  Generated: 2026-06-14 22:20:23   |   App URL: http://localhost:5173/CampusConnect_web/</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>871.4s</t>
+          <t>884.4s</t>
         </is>
       </c>
     </row>
@@ -1168,11 +1168,11 @@
         </is>
       </c>
       <c r="D4" s="23" t="n">
-        <v>3.196</v>
+        <v>3.089</v>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:02</t>
+          <t>2026-06-14 22:05:47</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -1196,11 +1196,11 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>4.211</v>
+        <v>4.215</v>
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:06</t>
+          <t>2026-06-14 22:05:51</t>
         </is>
       </c>
       <c r="F5" s="28" t="inlineStr">
@@ -1224,11 +1224,11 @@
         </is>
       </c>
       <c r="D6" s="23" t="n">
-        <v>4.367</v>
+        <v>4.391</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:10</t>
+          <t>2026-06-14 22:05:56</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -1252,11 +1252,11 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>4.363</v>
+        <v>4.667</v>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:15</t>
+          <t>2026-06-14 22:06:00</t>
         </is>
       </c>
       <c r="F7" s="28" t="inlineStr">
@@ -1280,11 +1280,11 @@
         </is>
       </c>
       <c r="D8" s="23" t="n">
-        <v>5.425</v>
+        <v>5.502</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:20</t>
+          <t>2026-06-14 22:06:06</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
@@ -1308,11 +1308,11 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>4.242</v>
+        <v>4.185</v>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:24</t>
+          <t>2026-06-14 22:06:10</t>
         </is>
       </c>
       <c r="F9" s="28" t="inlineStr">
@@ -1336,11 +1336,11 @@
         </is>
       </c>
       <c r="D10" s="23" t="n">
-        <v>4.297</v>
+        <v>4.284</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:29</t>
+          <t>2026-06-14 22:06:14</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
@@ -1364,11 +1364,11 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>6.402</v>
+        <v>6.379</v>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:35</t>
+          <t>2026-06-14 22:06:21</t>
         </is>
       </c>
       <c r="F11" s="28" t="inlineStr">
@@ -1392,16 +1392,16 @@
         </is>
       </c>
       <c r="D12" s="23" t="n">
-        <v>6.875</v>
+        <v>6.412</v>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:42</t>
+          <t>2026-06-14 22:06:27</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>Login with correct credentials succeeded. Redirected to 'http://localhost:5173/'.</t>
+          <t>Login with correct credentials succeeded. Redirected to 'http://localhost:5173/CampusConnect_web/#/'.</t>
         </is>
       </c>
     </row>
@@ -1420,11 +1420,11 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>5.158</v>
+        <v>5.093</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:47</t>
+          <t>2026-06-14 22:06:32</t>
         </is>
       </c>
       <c r="F13" s="28" t="inlineStr">
@@ -1448,11 +1448,11 @@
         </is>
       </c>
       <c r="D14" s="23" t="n">
-        <v>5.132</v>
+        <v>5.082</v>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:52</t>
+          <t>2026-06-14 22:06:37</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
@@ -1476,11 +1476,11 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5.14</v>
+        <v>5.118</v>
       </c>
       <c r="E15" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:41:57</t>
+          <t>2026-06-14 22:06:42</t>
         </is>
       </c>
       <c r="F15" s="28" t="inlineStr">
@@ -1504,11 +1504,11 @@
         </is>
       </c>
       <c r="D16" s="23" t="n">
-        <v>5.177</v>
+        <v>5.097</v>
       </c>
       <c r="E16" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:42:03</t>
+          <t>2026-06-14 22:06:48</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
@@ -1532,11 +1532,11 @@
         </is>
       </c>
       <c r="D17" s="27" t="n">
-        <v>8.318</v>
+        <v>8.223000000000001</v>
       </c>
       <c r="E17" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:42:11</t>
+          <t>2026-06-14 22:06:56</t>
         </is>
       </c>
       <c r="F17" s="28" t="inlineStr">
@@ -1560,11 +1560,11 @@
         </is>
       </c>
       <c r="D18" s="23" t="n">
-        <v>6.436</v>
+        <v>6.361</v>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:42:17</t>
+          <t>2026-06-14 22:07:02</t>
         </is>
       </c>
       <c r="F18" s="24" t="inlineStr">
@@ -1588,11 +1588,11 @@
         </is>
       </c>
       <c r="D19" s="27" t="n">
-        <v>5.201</v>
+        <v>5.138</v>
       </c>
       <c r="E19" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:55:10</t>
+          <t>2026-06-14 22:19:56</t>
         </is>
       </c>
       <c r="F19" s="28" t="inlineStr">
@@ -1616,11 +1616,11 @@
         </is>
       </c>
       <c r="D20" s="23" t="n">
-        <v>3.12</v>
+        <v>6.069</v>
       </c>
       <c r="E20" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:55:13</t>
+          <t>2026-06-14 22:20:02</t>
         </is>
       </c>
       <c r="F20" s="24" t="inlineStr">
@@ -1644,11 +1644,11 @@
         </is>
       </c>
       <c r="D21" s="27" t="n">
-        <v>3.116</v>
+        <v>6.063</v>
       </c>
       <c r="E21" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:55:16</t>
+          <t>2026-06-14 22:20:08</t>
         </is>
       </c>
       <c r="F21" s="28" t="inlineStr">
@@ -1672,11 +1672,11 @@
         </is>
       </c>
       <c r="D22" s="23" t="n">
-        <v>3.115</v>
+        <v>6.07</v>
       </c>
       <c r="E22" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:55:19</t>
+          <t>2026-06-14 22:20:14</t>
         </is>
       </c>
       <c r="F22" s="24" t="inlineStr">
@@ -1700,11 +1700,11 @@
         </is>
       </c>
       <c r="D23" s="27" t="n">
-        <v>3.118</v>
+        <v>6.06</v>
       </c>
       <c r="E23" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:55:22</t>
+          <t>2026-06-14 22:20:21</t>
         </is>
       </c>
       <c r="F23" s="28" t="inlineStr">
@@ -1822,11 +1822,11 @@
         </is>
       </c>
       <c r="D4" s="23" t="n">
-        <v>6.176</v>
+        <v>6.087</v>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:42:23</t>
+          <t>2026-06-14 22:07:08</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -1850,11 +1850,11 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>6.232</v>
+        <v>6.122</v>
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:42:30</t>
+          <t>2026-06-14 22:07:14</t>
         </is>
       </c>
       <c r="F5" s="28" t="inlineStr">
@@ -1878,11 +1878,11 @@
         </is>
       </c>
       <c r="D6" s="23" t="n">
-        <v>6.134</v>
+        <v>6.088</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:42:36</t>
+          <t>2026-06-14 22:07:20</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -1906,11 +1906,11 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>9.231999999999999</v>
+        <v>9.25</v>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:42:45</t>
+          <t>2026-06-14 22:07:30</t>
         </is>
       </c>
       <c r="F7" s="28" t="inlineStr">
@@ -1934,11 +1934,11 @@
         </is>
       </c>
       <c r="D8" s="23" t="n">
-        <v>11.352</v>
+        <v>11.329</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:42:56</t>
+          <t>2026-06-14 22:07:41</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
@@ -1962,11 +1962,11 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>11.272</v>
+        <v>11.2</v>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:43:08</t>
+          <t>2026-06-14 22:07:52</t>
         </is>
       </c>
       <c r="F9" s="28" t="inlineStr">
@@ -1990,16 +1990,16 @@
         </is>
       </c>
       <c r="D10" s="23" t="n">
-        <v>6.18</v>
+        <v>6.085</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:43:14</t>
+          <t>2026-06-14 22:07:58</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
         <is>
-          <t>Freelancer cards display names correctly. Found: API QA Engineer, Achyuth.</t>
+          <t>Freelancer cards display names correctly. Found: Achyuth.</t>
         </is>
       </c>
     </row>
@@ -2018,16 +2018,16 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>6.161</v>
+        <v>6.084</v>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:43:20</t>
+          <t>2026-06-14 22:08:04</t>
         </is>
       </c>
       <c r="F11" s="28" t="inlineStr">
         <is>
-          <t>Freelancer cards correctly display academic departments (e.g. 'Computer Science').</t>
+          <t>Freelancer cards correctly display academic departments (e.g. 'Computer science').</t>
         </is>
       </c>
     </row>
@@ -2046,16 +2046,16 @@
         </is>
       </c>
       <c r="D12" s="23" t="n">
-        <v>6.133</v>
+        <v>6.066</v>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:43:26</t>
+          <t>2026-06-14 22:08:10</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>Freelancer cards display skill chips correctly (3 chips found across all cards).</t>
+          <t>Freelancer cards display skill chips correctly (1 chips found across all cards).</t>
         </is>
       </c>
     </row>
@@ -2074,11 +2074,11 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>6.151</v>
+        <v>6.082</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:43:32</t>
+          <t>2026-06-14 22:08:17</t>
         </is>
       </c>
       <c r="F13" s="28" t="inlineStr">
@@ -2102,16 +2102,16 @@
         </is>
       </c>
       <c r="D14" s="23" t="n">
-        <v>9.189</v>
+        <v>9.137</v>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:43:42</t>
+          <t>2026-06-14 22:08:26</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>Clicking freelancer card navigated to profile page at 'http://localhost:5173/profile/AUV1reaQquP85Ya7oJ7zWgK4vED2'.</t>
+          <t>Clicking freelancer card navigated to profile page at 'http://localhost:5173/CampusConnect_web/#/profile/vAaAiqCoNYdo0MUyzIQSBL2AYvS2'.</t>
         </is>
       </c>
     </row>
@@ -2130,11 +2130,11 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>9.275</v>
+        <v>9.175000000000001</v>
       </c>
       <c r="E15" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:43:51</t>
+          <t>2026-06-14 22:08:35</t>
         </is>
       </c>
       <c r="F15" s="28" t="inlineStr">
@@ -2158,11 +2158,11 @@
         </is>
       </c>
       <c r="D16" s="23" t="n">
-        <v>9.196999999999999</v>
+        <v>9.132999999999999</v>
       </c>
       <c r="E16" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:44:00</t>
+          <t>2026-06-14 22:08:44</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
@@ -2186,11 +2186,11 @@
         </is>
       </c>
       <c r="D17" s="27" t="n">
-        <v>9.214</v>
+        <v>9.148999999999999</v>
       </c>
       <c r="E17" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:44:09</t>
+          <t>2026-06-14 22:08:53</t>
         </is>
       </c>
       <c r="F17" s="28" t="inlineStr">
@@ -2214,11 +2214,11 @@
         </is>
       </c>
       <c r="D18" s="23" t="n">
-        <v>11.19</v>
+        <v>11.152</v>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:44:20</t>
+          <t>2026-06-14 22:09:04</t>
         </is>
       </c>
       <c r="F18" s="24" t="inlineStr">
@@ -2331,11 +2331,11 @@
         </is>
       </c>
       <c r="D4" s="23" t="n">
-        <v>6.209</v>
+        <v>6.154</v>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:44:27</t>
+          <t>2026-06-14 22:09:10</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -2359,11 +2359,11 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>6.189</v>
+        <v>6.138</v>
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:44:33</t>
+          <t>2026-06-14 22:09:17</t>
         </is>
       </c>
       <c r="F5" s="28" t="inlineStr">
@@ -2387,11 +2387,11 @@
         </is>
       </c>
       <c r="D6" s="23" t="n">
-        <v>6.204</v>
+        <v>6.145</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:44:39</t>
+          <t>2026-06-14 22:09:23</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -2415,11 +2415,11 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>20.163</v>
+        <v>20.512</v>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:44:59</t>
+          <t>2026-06-14 22:09:43</t>
         </is>
       </c>
       <c r="F7" s="28" t="inlineStr">
@@ -2443,11 +2443,11 @@
         </is>
       </c>
       <c r="D8" s="23" t="n">
-        <v>8.228999999999999</v>
+        <v>8.151999999999999</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:45:07</t>
+          <t>2026-06-14 22:09:51</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
@@ -2471,11 +2471,11 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>8.196</v>
+        <v>8.128</v>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:45:16</t>
+          <t>2026-06-14 22:09:59</t>
         </is>
       </c>
       <c r="F9" s="28" t="inlineStr">
@@ -2499,11 +2499,11 @@
         </is>
       </c>
       <c r="D10" s="23" t="n">
-        <v>6.186</v>
+        <v>6.08</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:45:22</t>
+          <t>2026-06-14 22:10:06</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
@@ -2527,11 +2527,11 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>6.132</v>
+        <v>6.118</v>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:45:28</t>
+          <t>2026-06-14 22:10:12</t>
         </is>
       </c>
       <c r="F11" s="28" t="inlineStr">
@@ -2555,11 +2555,11 @@
         </is>
       </c>
       <c r="D12" s="23" t="n">
-        <v>6.132</v>
+        <v>6.068</v>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:45:34</t>
+          <t>2026-06-14 22:10:18</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
@@ -2583,11 +2583,11 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>6.147</v>
+        <v>6.088</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:45:40</t>
+          <t>2026-06-14 22:10:24</t>
         </is>
       </c>
       <c r="F13" s="28" t="inlineStr">
@@ -2611,11 +2611,11 @@
         </is>
       </c>
       <c r="D14" s="23" t="n">
-        <v>6.173</v>
+        <v>6.115</v>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:45:46</t>
+          <t>2026-06-14 22:10:30</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
@@ -2639,11 +2639,11 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>6.151</v>
+        <v>6.096</v>
       </c>
       <c r="E15" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:45:53</t>
+          <t>2026-06-14 22:10:36</t>
         </is>
       </c>
       <c r="F15" s="28" t="inlineStr">
@@ -2667,11 +2667,11 @@
         </is>
       </c>
       <c r="D16" s="23" t="n">
-        <v>6.147</v>
+        <v>6.102</v>
       </c>
       <c r="E16" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:45:59</t>
+          <t>2026-06-14 22:10:42</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
@@ -2695,11 +2695,11 @@
         </is>
       </c>
       <c r="D17" s="27" t="n">
-        <v>8.231999999999999</v>
+        <v>8.154</v>
       </c>
       <c r="E17" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:46:07</t>
+          <t>2026-06-14 22:10:50</t>
         </is>
       </c>
       <c r="F17" s="28" t="inlineStr">
@@ -2723,11 +2723,11 @@
         </is>
       </c>
       <c r="D18" s="23" t="n">
-        <v>14.737</v>
+        <v>14.862</v>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:46:22</t>
+          <t>2026-06-14 22:11:05</t>
         </is>
       </c>
       <c r="F18" s="24" t="inlineStr">
@@ -2751,11 +2751,11 @@
         </is>
       </c>
       <c r="D19" s="27" t="n">
-        <v>6.326</v>
+        <v>6.218</v>
       </c>
       <c r="E19" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:46:28</t>
+          <t>2026-06-14 22:11:11</t>
         </is>
       </c>
       <c r="F19" s="28" t="inlineStr">
@@ -2779,16 +2779,16 @@
         </is>
       </c>
       <c r="D20" s="23" t="n">
-        <v>9.222</v>
+        <v>9.183</v>
       </c>
       <c r="E20" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:46:37</t>
+          <t>2026-06-14 22:11:21</t>
         </is>
       </c>
       <c r="F20" s="24" t="inlineStr">
         <is>
-          <t>Clicking gig card navigated to detail page at 'http://localhost:5173/gigs/a6diJnso1NZYnERqDp75'.</t>
+          <t>Clicking gig card navigated to detail page at 'http://localhost:5173/CampusConnect_web/#/gigs/mChZqyYPKy9aI6GGBdFe'.</t>
         </is>
       </c>
     </row>
@@ -2807,11 +2807,11 @@
         </is>
       </c>
       <c r="D21" s="27" t="n">
-        <v>9.222</v>
+        <v>9.161</v>
       </c>
       <c r="E21" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:46:46</t>
+          <t>2026-06-14 22:11:30</t>
         </is>
       </c>
       <c r="F21" s="28" t="inlineStr">
@@ -2835,11 +2835,11 @@
         </is>
       </c>
       <c r="D22" s="23" t="n">
-        <v>8.151</v>
+        <v>8.106999999999999</v>
       </c>
       <c r="E22" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:46:55</t>
+          <t>2026-06-14 22:11:38</t>
         </is>
       </c>
       <c r="F22" s="24" t="inlineStr">
@@ -2863,11 +2863,11 @@
         </is>
       </c>
       <c r="D23" s="27" t="n">
-        <v>9.16</v>
+        <v>9.124000000000001</v>
       </c>
       <c r="E23" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:47:04</t>
+          <t>2026-06-14 22:11:47</t>
         </is>
       </c>
       <c r="F23" s="28" t="inlineStr">
@@ -2985,11 +2985,11 @@
         </is>
       </c>
       <c r="D4" s="23" t="n">
-        <v>6.154</v>
+        <v>6.098</v>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:47:10</t>
+          <t>2026-06-14 22:11:53</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -3013,11 +3013,11 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>6.153</v>
+        <v>6.083</v>
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:47:16</t>
+          <t>2026-06-14 22:11:59</t>
         </is>
       </c>
       <c r="F5" s="28" t="inlineStr">
@@ -3041,11 +3041,11 @@
         </is>
       </c>
       <c r="D6" s="23" t="n">
-        <v>6.148</v>
+        <v>6.085</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:47:22</t>
+          <t>2026-06-14 22:12:05</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -3069,11 +3069,11 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>8.346</v>
+        <v>8.196999999999999</v>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:47:31</t>
+          <t>2026-06-14 22:12:13</t>
         </is>
       </c>
       <c r="F7" s="28" t="inlineStr">
@@ -3097,11 +3097,11 @@
         </is>
       </c>
       <c r="D8" s="23" t="n">
-        <v>8.239000000000001</v>
+        <v>9.161</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:47:39</t>
+          <t>2026-06-14 22:12:23</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
@@ -3125,11 +3125,11 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>10.268</v>
+        <v>11.19</v>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:47:49</t>
+          <t>2026-06-14 22:12:34</t>
         </is>
       </c>
       <c r="F9" s="28" t="inlineStr">
@@ -3153,11 +3153,11 @@
         </is>
       </c>
       <c r="D10" s="23" t="n">
-        <v>10.32</v>
+        <v>11.278</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:47:59</t>
+          <t>2026-06-14 22:12:45</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
@@ -3181,16 +3181,16 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>15.57</v>
+        <v>16.582</v>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:48:15</t>
+          <t>2026-06-14 22:13:02</t>
         </is>
       </c>
       <c r="F11" s="28" t="inlineStr">
         <is>
-          <t>Team 'E2E Squad 3525' created successfully with 'React' skill via the Create Team form.</t>
+          <t>Team 'E2E Squad 3CBD' created successfully with 'React' skill via the Create Team form.</t>
         </is>
       </c>
     </row>
@@ -3209,16 +3209,16 @@
         </is>
       </c>
       <c r="D12" s="23" t="n">
-        <v>6.185</v>
+        <v>6.177</v>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:48:21</t>
+          <t>2026-06-14 22:13:08</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>Teams listing shows created teams (6 team cards found).</t>
+          <t>Teams listing shows created teams (7 team cards found).</t>
         </is>
       </c>
     </row>
@@ -3237,11 +3237,11 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>6.267</v>
+        <v>6.251</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:48:27</t>
+          <t>2026-06-14 22:13:14</t>
         </is>
       </c>
       <c r="F13" s="28" t="inlineStr">
@@ -3265,11 +3265,11 @@
         </is>
       </c>
       <c r="D14" s="23" t="n">
-        <v>6.137</v>
+        <v>6.115</v>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:48:33</t>
+          <t>2026-06-14 22:13:20</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
@@ -3293,11 +3293,11 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>8.196999999999999</v>
+        <v>8.159000000000001</v>
       </c>
       <c r="E15" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:48:42</t>
+          <t>2026-06-14 22:13:28</t>
         </is>
       </c>
       <c r="F15" s="28" t="inlineStr">
@@ -3321,11 +3321,11 @@
         </is>
       </c>
       <c r="D16" s="23" t="n">
-        <v>8.198</v>
+        <v>8.138</v>
       </c>
       <c r="E16" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:48:50</t>
+          <t>2026-06-14 22:13:36</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
@@ -3349,11 +3349,11 @@
         </is>
       </c>
       <c r="D17" s="27" t="n">
-        <v>8.231</v>
+        <v>8.144</v>
       </c>
       <c r="E17" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:48:58</t>
+          <t>2026-06-14 22:13:45</t>
         </is>
       </c>
       <c r="F17" s="28" t="inlineStr">
@@ -3377,11 +3377,11 @@
         </is>
       </c>
       <c r="D18" s="23" t="n">
-        <v>8.27</v>
+        <v>8.119</v>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:49:06</t>
+          <t>2026-06-14 22:13:53</t>
         </is>
       </c>
       <c r="F18" s="24" t="inlineStr">
@@ -3494,11 +3494,11 @@
         </is>
       </c>
       <c r="D4" s="23" t="n">
-        <v>6.129</v>
+        <v>6.108</v>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:50:30</t>
+          <t>2026-06-14 22:15:16</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -3522,11 +3522,11 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>6.16</v>
+        <v>6.074</v>
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:50:36</t>
+          <t>2026-06-14 22:15:22</t>
         </is>
       </c>
       <c r="F5" s="28" t="inlineStr">
@@ -3550,11 +3550,11 @@
         </is>
       </c>
       <c r="D6" s="23" t="n">
-        <v>8.109999999999999</v>
+        <v>8.025</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:50:44</t>
+          <t>2026-06-14 22:15:30</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -3578,11 +3578,11 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>8.096</v>
+        <v>8.032</v>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:50:52</t>
+          <t>2026-06-14 22:15:38</t>
         </is>
       </c>
       <c r="F7" s="28" t="inlineStr">
@@ -3606,11 +3606,11 @@
         </is>
       </c>
       <c r="D8" s="23" t="n">
-        <v>6.144</v>
+        <v>6.094</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:50:59</t>
+          <t>2026-06-14 22:15:44</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
@@ -3634,11 +3634,11 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>8.093</v>
+        <v>8.041</v>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:51:07</t>
+          <t>2026-06-14 22:15:52</t>
         </is>
       </c>
       <c r="F9" s="28" t="inlineStr">
@@ -3662,11 +3662,11 @@
         </is>
       </c>
       <c r="D10" s="23" t="n">
-        <v>8.090999999999999</v>
+        <v>8.039</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:51:15</t>
+          <t>2026-06-14 22:16:00</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
@@ -3690,11 +3690,11 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>8.112</v>
+        <v>8.044</v>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:51:23</t>
+          <t>2026-06-14 22:16:08</t>
         </is>
       </c>
       <c r="F11" s="28" t="inlineStr">
@@ -3718,11 +3718,11 @@
         </is>
       </c>
       <c r="D12" s="23" t="n">
-        <v>10.115</v>
+        <v>10.033</v>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:51:33</t>
+          <t>2026-06-14 22:16:18</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
@@ -3746,11 +3746,11 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>10.223</v>
+        <v>10.134</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:51:43</t>
+          <t>2026-06-14 22:16:28</t>
         </is>
       </c>
       <c r="F13" s="28" t="inlineStr">
@@ -3774,11 +3774,11 @@
         </is>
       </c>
       <c r="D14" s="23" t="n">
-        <v>8.109</v>
+        <v>8.032999999999999</v>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:51:51</t>
+          <t>2026-06-14 22:16:36</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
@@ -3802,11 +3802,11 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>17.285</v>
+        <v>17.148</v>
       </c>
       <c r="E15" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:52:09</t>
+          <t>2026-06-14 22:16:53</t>
         </is>
       </c>
       <c r="F15" s="28" t="inlineStr">
@@ -3830,11 +3830,11 @@
         </is>
       </c>
       <c r="D16" s="23" t="n">
-        <v>12.264</v>
+        <v>12.22</v>
       </c>
       <c r="E16" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:52:21</t>
+          <t>2026-06-14 22:17:06</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
@@ -3945,11 +3945,11 @@
         </is>
       </c>
       <c r="D4" s="23" t="n">
-        <v>7.245</v>
+        <v>7.216</v>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:49:14</t>
+          <t>2026-06-14 22:14:00</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -3973,11 +3973,11 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>7.239</v>
+        <v>7.18</v>
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:49:21</t>
+          <t>2026-06-14 22:14:07</t>
         </is>
       </c>
       <c r="F5" s="28" t="inlineStr">
@@ -4001,11 +4001,11 @@
         </is>
       </c>
       <c r="D6" s="23" t="n">
-        <v>7.264</v>
+        <v>7.197</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:49:28</t>
+          <t>2026-06-14 22:14:14</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -4029,11 +4029,11 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>7.271</v>
+        <v>7.201</v>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:49:35</t>
+          <t>2026-06-14 22:14:22</t>
         </is>
       </c>
       <c r="F7" s="28" t="inlineStr">
@@ -4057,11 +4057,11 @@
         </is>
       </c>
       <c r="D8" s="23" t="n">
-        <v>7.257</v>
+        <v>7.181</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:49:43</t>
+          <t>2026-06-14 22:14:29</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
@@ -4085,11 +4085,11 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>7.236</v>
+        <v>7.184</v>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:49:50</t>
+          <t>2026-06-14 22:14:36</t>
         </is>
       </c>
       <c r="F9" s="28" t="inlineStr">
@@ -4113,11 +4113,11 @@
         </is>
       </c>
       <c r="D10" s="23" t="n">
-        <v>7.264</v>
+        <v>7.198</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:49:57</t>
+          <t>2026-06-14 22:14:43</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
@@ -4141,11 +4141,11 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>7.27</v>
+        <v>7.19</v>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:50:04</t>
+          <t>2026-06-14 22:14:50</t>
         </is>
       </c>
       <c r="F11" s="28" t="inlineStr">
@@ -4169,11 +4169,11 @@
         </is>
       </c>
       <c r="D12" s="23" t="n">
-        <v>19.465</v>
+        <v>19.293</v>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:50:24</t>
+          <t>2026-06-14 22:15:10</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
@@ -4280,11 +4280,11 @@
         </is>
       </c>
       <c r="D4" s="23" t="n">
-        <v>6.164</v>
+        <v>6.102</v>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:52:27</t>
+          <t>2026-06-14 22:17:12</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -4308,11 +4308,11 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>6.163</v>
+        <v>6.118</v>
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:52:33</t>
+          <t>2026-06-14 22:17:18</t>
         </is>
       </c>
       <c r="F5" s="28" t="inlineStr">
@@ -4336,11 +4336,11 @@
         </is>
       </c>
       <c r="D6" s="23" t="n">
-        <v>6.144</v>
+        <v>6.099</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:52:39</t>
+          <t>2026-06-14 22:17:24</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -4364,11 +4364,11 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>6.132</v>
+        <v>6.099</v>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:52:45</t>
+          <t>2026-06-14 22:17:30</t>
         </is>
       </c>
       <c r="F7" s="28" t="inlineStr">
@@ -4392,11 +4392,11 @@
         </is>
       </c>
       <c r="D8" s="23" t="n">
-        <v>6.148</v>
+        <v>6.116</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:52:52</t>
+          <t>2026-06-14 22:17:36</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
@@ -4420,11 +4420,11 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>6.154</v>
+        <v>6.103</v>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:52:58</t>
+          <t>2026-06-14 22:17:42</t>
         </is>
       </c>
       <c r="F9" s="28" t="inlineStr">
@@ -4448,11 +4448,11 @@
         </is>
       </c>
       <c r="D10" s="23" t="n">
-        <v>8.220000000000001</v>
+        <v>8.151999999999999</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:53:06</t>
+          <t>2026-06-14 22:17:50</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
@@ -4476,11 +4476,11 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>6.156</v>
+        <v>6.089</v>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:53:12</t>
+          <t>2026-06-14 22:17:56</t>
         </is>
       </c>
       <c r="F11" s="28" t="inlineStr">
@@ -4504,11 +4504,11 @@
         </is>
       </c>
       <c r="D12" s="23" t="n">
-        <v>8.167</v>
+        <v>8.119</v>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:53:20</t>
+          <t>2026-06-14 22:18:05</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
@@ -4532,11 +4532,11 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>9.199</v>
+        <v>9.132999999999999</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:53:29</t>
+          <t>2026-06-14 22:18:14</t>
         </is>
       </c>
       <c r="F13" s="28" t="inlineStr">
@@ -4560,11 +4560,11 @@
         </is>
       </c>
       <c r="D14" s="23" t="n">
-        <v>11.289</v>
+        <v>11.195</v>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:53:41</t>
+          <t>2026-06-14 22:18:25</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
@@ -4588,11 +4588,11 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5.137</v>
+        <v>5.09</v>
       </c>
       <c r="E15" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:53:46</t>
+          <t>2026-06-14 22:18:30</t>
         </is>
       </c>
       <c r="F15" s="28" t="inlineStr">
@@ -4616,11 +4616,11 @@
         </is>
       </c>
       <c r="D16" s="23" t="n">
-        <v>9.193</v>
+        <v>9.129</v>
       </c>
       <c r="E16" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:53:55</t>
+          <t>2026-06-14 22:18:39</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
@@ -4731,11 +4731,11 @@
         </is>
       </c>
       <c r="D4" s="23" t="n">
-        <v>6.197</v>
+        <v>6.106</v>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:54:01</t>
+          <t>2026-06-14 22:18:45</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -4759,11 +4759,11 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>6.161</v>
+        <v>6.083</v>
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:54:07</t>
+          <t>2026-06-14 22:18:51</t>
         </is>
       </c>
       <c r="F5" s="28" t="inlineStr">
@@ -4787,11 +4787,11 @@
         </is>
       </c>
       <c r="D6" s="23" t="n">
-        <v>6.144</v>
+        <v>6.097</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:54:14</t>
+          <t>2026-06-14 22:18:57</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -4815,11 +4815,11 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>6.149</v>
+        <v>6.097</v>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:54:20</t>
+          <t>2026-06-14 22:19:04</t>
         </is>
       </c>
       <c r="F7" s="28" t="inlineStr">
@@ -4843,11 +4843,11 @@
         </is>
       </c>
       <c r="D8" s="23" t="n">
-        <v>6.144</v>
+        <v>6.089</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:54:26</t>
+          <t>2026-06-14 22:19:10</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
@@ -4871,11 +4871,11 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>6.161</v>
+        <v>6.089</v>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:54:32</t>
+          <t>2026-06-14 22:19:16</t>
         </is>
       </c>
       <c r="F9" s="28" t="inlineStr">
@@ -4899,11 +4899,11 @@
         </is>
       </c>
       <c r="D10" s="23" t="n">
-        <v>6.18</v>
+        <v>6.092</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:54:38</t>
+          <t>2026-06-14 22:19:22</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
@@ -4927,11 +4927,11 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>6.123</v>
+        <v>6.084</v>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:54:44</t>
+          <t>2026-06-14 22:19:28</t>
         </is>
       </c>
       <c r="F11" s="28" t="inlineStr">
@@ -4955,11 +4955,11 @@
         </is>
       </c>
       <c r="D12" s="23" t="n">
-        <v>3.155</v>
+        <v>6.109</v>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>2026-06-11 14:54:48</t>
+          <t>2026-06-14 22:19:34</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
@@ -4983,16 +4983,16 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>17.305</v>
+        <v>17.139</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>2026-06-11 14:55:05</t>
+          <t>2026-06-14 22:19:51</t>
         </is>
       </c>
       <c r="F13" s="28" t="inlineStr">
         <is>
-          <t>Browser back button correctly navigated to the previous page: 'http://localhost:5173/gigs'.</t>
+          <t>Browser back button correctly navigated to the previous page: 'http://localhost:5173/CampusConnect_web/#/gigs'.</t>
         </is>
       </c>
     </row>

</xml_diff>